<commit_message>
Updated BOM and print file.
</commit_message>
<xml_diff>
--- a/Active Pedal BOM.xlsx
+++ b/Active Pedal BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\source\zfgffb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6AF9CA3E-B04E-4B1C-AC19-97F4668825E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A63D2B9-5383-4989-B80A-0BE98734A44B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7890" yWindow="2340" windowWidth="28155" windowHeight="17895" activeTab="1" xr2:uid="{7B48C4A4-57E3-4029-9556-E0999BF8FA96}"/>
+    <workbookView xWindow="7890" yWindow="2340" windowWidth="28155" windowHeight="17895" xr2:uid="{7B48C4A4-57E3-4029-9556-E0999BF8FA96}"/>
   </bookViews>
   <sheets>
     <sheet name="Group Buy" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="160">
   <si>
     <t>Chris</t>
   </si>
@@ -501,6 +501,24 @@
   </si>
   <si>
     <t>Tolerances were tight for me and this came in handy more than once.</t>
+  </si>
+  <si>
+    <t>M6</t>
+  </si>
+  <si>
+    <t>M6 Nuts</t>
+  </si>
+  <si>
+    <t>M6 Washers</t>
+  </si>
+  <si>
+    <t>Fasteners</t>
+  </si>
+  <si>
+    <t>M6x???</t>
+  </si>
+  <si>
+    <t>Length depends on your mounting plate.  22.3mm is the length needed to reach the bottom of the plate.  Add length as necessary.</t>
   </si>
 </sst>
 </file>
@@ -545,11 +563,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -899,7 +920,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1D4D29E-CC41-4B87-BDEC-C4346A654BBE}">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -941,7 +962,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>71</v>
       </c>
       <c r="B2" t="s">
@@ -954,11 +975,11 @@
         <v>50</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E33" si="0">C2*$C$36</f>
+        <f>C2*$C$38</f>
         <v>14</v>
       </c>
       <c r="F2">
-        <f t="shared" ref="F2:F11" si="1">ROUNDUP(E2/D2,0)</f>
+        <f t="shared" ref="F2:F11" si="0">ROUNDUP(E2/D2,0)</f>
         <v>1</v>
       </c>
       <c r="G2">
@@ -969,12 +990,12 @@
         <v>7.29</v>
       </c>
       <c r="I2">
-        <f>ROUNDDOWN(D2*F2/$C$36, 0)</f>
+        <f>ROUNDDOWN(D2*F2/$C$38, 0)</f>
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
+      <c r="A3" s="5"/>
       <c r="B3" t="s">
         <v>11</v>
       </c>
@@ -985,27 +1006,27 @@
         <v>100</v>
       </c>
       <c r="E3">
+        <f>C3*$C$38</f>
+        <v>105</v>
+      </c>
+      <c r="F3">
         <f t="shared" si="0"/>
-        <v>105</v>
-      </c>
-      <c r="F3">
-        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="G3">
         <v>8.69</v>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H34" si="2">G3*F3</f>
+        <f t="shared" ref="H3:H36" si="1">G3*F3</f>
         <v>17.38</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I33" si="3">ROUNDDOWN(D3*F3/$C$36, 0)</f>
+        <f>ROUNDDOWN(D3*F3/$C$38, 0)</f>
         <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
+      <c r="A4" s="5"/>
       <c r="B4" t="s">
         <v>25</v>
       </c>
@@ -1016,27 +1037,27 @@
         <v>120</v>
       </c>
       <c r="E4">
+        <f>C4*$C$38</f>
+        <v>28</v>
+      </c>
+      <c r="F4">
         <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="F4">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G4">
         <v>7.99</v>
       </c>
       <c r="H4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7.99</v>
       </c>
       <c r="I4">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D4*F4/$C$38, 0)</f>
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
+      <c r="A5" s="5"/>
       <c r="B5" t="s">
         <v>26</v>
       </c>
@@ -1047,27 +1068,27 @@
         <v>100</v>
       </c>
       <c r="E5">
+        <f>C5*$C$38</f>
+        <v>14</v>
+      </c>
+      <c r="F5">
         <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="F5">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G5">
         <v>6.96</v>
       </c>
       <c r="H5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>6.96</v>
       </c>
       <c r="I5">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D5*F5/$C$38, 0)</f>
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
+      <c r="A6" s="5"/>
       <c r="B6" t="s">
         <v>49</v>
       </c>
@@ -1078,27 +1099,27 @@
         <v>100</v>
       </c>
       <c r="E6">
+        <f>C6*$C$38</f>
+        <v>42</v>
+      </c>
+      <c r="F6">
         <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="F6">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G6">
         <v>8.2799999999999994</v>
       </c>
       <c r="H6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8.2799999999999994</v>
       </c>
       <c r="I6">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D6*F6/$C$38, 0)</f>
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
+      <c r="A7" s="5"/>
       <c r="B7" t="s">
         <v>12</v>
       </c>
@@ -1109,27 +1130,27 @@
         <v>100</v>
       </c>
       <c r="E7">
+        <f>C7*$C$38</f>
+        <v>28</v>
+      </c>
+      <c r="F7">
         <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="F7">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G7">
         <v>8.2799999999999994</v>
       </c>
       <c r="H7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8.2799999999999994</v>
       </c>
       <c r="I7">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D7*F7/$C$38, 0)</f>
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
+      <c r="A8" s="5"/>
       <c r="B8" t="s">
         <v>13</v>
       </c>
@@ -1140,27 +1161,27 @@
         <v>50</v>
       </c>
       <c r="E8">
+        <f>C8*$C$38</f>
+        <v>14</v>
+      </c>
+      <c r="F8">
         <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="F8">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G8">
         <v>7.59</v>
       </c>
       <c r="H8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7.59</v>
       </c>
       <c r="I8">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D8*F8/$C$38, 0)</f>
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
+      <c r="A9" s="5"/>
       <c r="B9" t="s">
         <v>48</v>
       </c>
@@ -1171,27 +1192,27 @@
         <v>100</v>
       </c>
       <c r="E9">
+        <f>C9*$C$38</f>
+        <v>7</v>
+      </c>
+      <c r="F9">
         <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G9">
         <v>8.68</v>
       </c>
       <c r="H9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8.68</v>
       </c>
       <c r="I9">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D9*F9/$C$38, 0)</f>
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
+      <c r="A10" s="5"/>
       <c r="B10" t="s">
         <v>51</v>
       </c>
@@ -1202,27 +1223,27 @@
         <v>200</v>
       </c>
       <c r="E10">
+        <f>C10*$C$38</f>
+        <v>14</v>
+      </c>
+      <c r="F10">
         <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G10">
         <v>6.99</v>
       </c>
       <c r="H10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>6.99</v>
       </c>
       <c r="I10">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D10*F10/$C$38, 0)</f>
         <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
+      <c r="A11" s="5"/>
       <c r="B11" t="s">
         <v>52</v>
       </c>
@@ -1233,27 +1254,27 @@
         <v>100</v>
       </c>
       <c r="E11">
+        <f>C11*$C$38</f>
+        <v>14</v>
+      </c>
+      <c r="F11">
         <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="F11">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G11">
         <v>7.69</v>
       </c>
       <c r="H11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7.69</v>
       </c>
       <c r="I11">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D11*F11/$C$38, 0)</f>
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="5" t="s">
         <v>72</v>
       </c>
       <c r="B12" t="s">
@@ -1266,27 +1287,27 @@
         <v>50</v>
       </c>
       <c r="E12">
-        <f t="shared" si="0"/>
+        <f>C12*$C$38</f>
         <v>84</v>
       </c>
       <c r="F12">
-        <f t="shared" ref="F12:F33" si="4">ROUNDUP(E12/D12,0)</f>
+        <f t="shared" ref="F12:F35" si="2">ROUNDUP(E12/D12,0)</f>
         <v>2</v>
       </c>
       <c r="G12">
         <v>9.99</v>
       </c>
       <c r="H12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>19.98</v>
       </c>
       <c r="I12">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D12*F12/$C$38, 0)</f>
         <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
+      <c r="A13" s="5"/>
       <c r="B13" t="s">
         <v>53</v>
       </c>
@@ -1297,27 +1318,27 @@
         <v>50</v>
       </c>
       <c r="E13">
-        <f t="shared" si="0"/>
+        <f>C13*$C$38</f>
         <v>14</v>
       </c>
       <c r="F13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G13">
         <v>7.99</v>
       </c>
       <c r="H13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7.99</v>
       </c>
       <c r="I13">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D13*F13/$C$38, 0)</f>
         <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
+      <c r="A14" s="5"/>
       <c r="B14" t="s">
         <v>54</v>
       </c>
@@ -1328,27 +1349,27 @@
         <v>100</v>
       </c>
       <c r="E14">
-        <f t="shared" si="0"/>
+        <f>C14*$C$38</f>
         <v>112</v>
       </c>
       <c r="F14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="G14">
         <v>9.49</v>
       </c>
       <c r="H14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>18.98</v>
       </c>
       <c r="I14">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D14*F14/$C$38, 0)</f>
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
+      <c r="A15" s="5"/>
       <c r="B15" t="s">
         <v>41</v>
       </c>
@@ -1359,7 +1380,7 @@
         <v>100</v>
       </c>
       <c r="E15">
-        <f t="shared" si="0"/>
+        <f>C15*$C$38</f>
         <v>28</v>
       </c>
       <c r="F15">
@@ -1370,16 +1391,16 @@
         <v>5.69</v>
       </c>
       <c r="H15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>5.69</v>
       </c>
       <c r="I15">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D15*F15/$C$38, 0)</f>
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
+      <c r="A16" s="5"/>
       <c r="B16" t="s">
         <v>42</v>
       </c>
@@ -1390,7 +1411,7 @@
         <v>120</v>
       </c>
       <c r="E16">
-        <f t="shared" si="0"/>
+        <f>C16*$C$38</f>
         <v>14</v>
       </c>
       <c r="F16">
@@ -1401,16 +1422,16 @@
         <v>8.99</v>
       </c>
       <c r="H16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8.99</v>
       </c>
       <c r="I16">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D16*F16/$C$38, 0)</f>
         <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="4"/>
+      <c r="A17" s="5"/>
       <c r="B17" t="s">
         <v>14</v>
       </c>
@@ -1421,7 +1442,7 @@
         <v>50</v>
       </c>
       <c r="E17">
-        <f t="shared" si="0"/>
+        <f>C17*$C$38</f>
         <v>70</v>
       </c>
       <c r="F17">
@@ -1432,16 +1453,16 @@
         <v>6.89</v>
       </c>
       <c r="H17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>13.78</v>
       </c>
       <c r="I17">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D17*F17/$C$38, 0)</f>
         <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
+      <c r="A18" s="5"/>
       <c r="B18" t="s">
         <v>43</v>
       </c>
@@ -1452,7 +1473,7 @@
         <v>50</v>
       </c>
       <c r="E18">
-        <f t="shared" si="0"/>
+        <f>C18*$C$38</f>
         <v>14</v>
       </c>
       <c r="F18">
@@ -1463,16 +1484,16 @@
         <v>8.4600000000000009</v>
       </c>
       <c r="H18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8.4600000000000009</v>
       </c>
       <c r="I18">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D18*F18/$C$38, 0)</f>
         <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>73</v>
       </c>
       <c r="B19" t="s">
@@ -1485,7 +1506,7 @@
         <v>50</v>
       </c>
       <c r="E19">
-        <f t="shared" si="0"/>
+        <f>C19*$C$38</f>
         <v>14</v>
       </c>
       <c r="F19">
@@ -1496,16 +1517,16 @@
         <v>8.86</v>
       </c>
       <c r="H19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8.86</v>
       </c>
       <c r="I19">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D19*F19/$C$38, 0)</f>
         <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="4"/>
+      <c r="A20" s="5"/>
       <c r="B20" t="s">
         <v>28</v>
       </c>
@@ -1516,27 +1537,27 @@
         <v>200</v>
       </c>
       <c r="E20">
-        <f t="shared" si="0"/>
+        <f>C20*$C$38</f>
         <v>0</v>
       </c>
       <c r="F20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G20">
         <v>9.99</v>
       </c>
       <c r="H20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I20">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D20*F20/$C$38, 0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="4"/>
+      <c r="A21" s="5"/>
       <c r="B21" t="s">
         <v>56</v>
       </c>
@@ -1547,27 +1568,27 @@
         <v>30</v>
       </c>
       <c r="E21">
-        <f t="shared" si="0"/>
+        <f>C21*$C$38</f>
         <v>28</v>
       </c>
       <c r="F21">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G21">
         <v>8.11</v>
       </c>
       <c r="H21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8.11</v>
       </c>
       <c r="I21">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D21*F21/$C$38, 0)</f>
         <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="4"/>
+      <c r="A22" s="5"/>
       <c r="B22" t="s">
         <v>29</v>
       </c>
@@ -1578,27 +1599,27 @@
         <v>50</v>
       </c>
       <c r="E22">
-        <f t="shared" si="0"/>
+        <f>C22*$C$38</f>
         <v>42</v>
       </c>
       <c r="F22">
-        <f t="shared" ref="F22:F28" si="5">ROUNDUP(E22/D22,0)</f>
+        <f t="shared" ref="F22:F30" si="3">ROUNDUP(E22/D22,0)</f>
         <v>1</v>
       </c>
       <c r="G22">
         <v>9.99</v>
       </c>
       <c r="H22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>9.99</v>
       </c>
       <c r="I22">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D22*F22/$C$38, 0)</f>
         <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="4"/>
+      <c r="A23" s="5"/>
       <c r="B23" t="s">
         <v>55</v>
       </c>
@@ -1609,27 +1630,27 @@
         <v>50</v>
       </c>
       <c r="E23">
-        <f t="shared" si="0"/>
+        <f>C23*$C$38</f>
         <v>14</v>
       </c>
       <c r="F23">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G23">
         <v>8.9600000000000009</v>
       </c>
       <c r="H23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8.9600000000000009</v>
       </c>
       <c r="I23">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D23*F23/$C$38, 0)</f>
         <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="4"/>
+      <c r="A24" s="5"/>
       <c r="B24" t="s">
         <v>57</v>
       </c>
@@ -1640,27 +1661,27 @@
         <v>25</v>
       </c>
       <c r="E24">
-        <f t="shared" si="0"/>
+        <f>C24*$C$38</f>
         <v>14</v>
       </c>
       <c r="F24">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G24">
         <v>7.99</v>
       </c>
       <c r="H24">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>7.99</v>
       </c>
       <c r="I24">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D24*F24/$C$38, 0)</f>
         <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="4"/>
+      <c r="A25" s="5"/>
       <c r="B25" t="s">
         <v>38</v>
       </c>
@@ -1671,124 +1692,126 @@
         <v>50</v>
       </c>
       <c r="E25">
-        <f t="shared" si="0"/>
+        <f>C25*$C$38</f>
         <v>14</v>
       </c>
       <c r="F25">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G25">
         <v>8.2799999999999994</v>
       </c>
       <c r="H25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>8.2799999999999994</v>
       </c>
       <c r="I25">
-        <f t="shared" si="3"/>
+        <f>ROUNDDOWN(D25*F25/$C$38, 0)</f>
         <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="4"/>
+      <c r="A26" s="5"/>
       <c r="B26" t="s">
         <v>39</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D26">
+        <v>30</v>
+      </c>
+      <c r="E26">
+        <f>C26*$C$38</f>
+        <v>14</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>9.99</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="1"/>
+        <v>9.99</v>
+      </c>
+      <c r="I26">
+        <f>ROUNDDOWN(D26*F26/$C$38, 0)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B27" t="s">
+        <v>155</v>
+      </c>
+      <c r="C27">
+        <v>6</v>
+      </c>
+      <c r="D27">
+        <v>50</v>
+      </c>
+      <c r="E27">
+        <f>C27*$C$38</f>
+        <v>42</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>6.19</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="1"/>
+        <v>6.19</v>
+      </c>
+      <c r="I27">
+        <f>ROUNDDOWN(D27*F27/$C$38, 0)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="3"/>
+      <c r="B28" t="s">
+        <v>156</v>
+      </c>
+      <c r="C28">
+        <v>6</v>
+      </c>
+      <c r="D28">
         <v>100</v>
       </c>
-      <c r="E26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F26">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="G26">
-        <v>0</v>
-      </c>
-      <c r="H26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I26">
+      <c r="E28">
+        <f>C28*$C$38</f>
+        <v>42</v>
+      </c>
+      <c r="F28">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G28">
+        <v>5.19</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="1"/>
+        <v>5.19</v>
+      </c>
+      <c r="I28">
+        <f>ROUNDDOWN(D28*F28/$C$38, 0)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B29" t="s">
         <v>37</v>
-      </c>
-      <c r="C27">
-        <v>2</v>
-      </c>
-      <c r="D27">
-        <v>20</v>
-      </c>
-      <c r="E27">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="F27">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-      <c r="G27">
-        <v>5.99</v>
-      </c>
-      <c r="H27">
-        <f t="shared" si="2"/>
-        <v>5.99</v>
-      </c>
-      <c r="I27">
-        <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="4"/>
-      <c r="B28" t="s">
-        <v>58</v>
-      </c>
-      <c r="C28">
-        <v>2</v>
-      </c>
-      <c r="D28">
-        <v>30</v>
-      </c>
-      <c r="E28">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="F28">
-        <f t="shared" si="5"/>
-        <v>1</v>
-      </c>
-      <c r="G28">
-        <v>8.5399999999999991</v>
-      </c>
-      <c r="H28">
-        <f t="shared" si="2"/>
-        <v>8.5399999999999991</v>
-      </c>
-      <c r="I28">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="4"/>
-      <c r="B29" t="s">
-        <v>59</v>
       </c>
       <c r="C29">
         <v>2</v>
@@ -1797,227 +1820,289 @@
         <v>20</v>
       </c>
       <c r="E29">
-        <f t="shared" si="0"/>
+        <f>C29*$C$38</f>
         <v>14</v>
       </c>
       <c r="F29">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="G29">
-        <v>8.99</v>
+        <v>5.99</v>
       </c>
       <c r="H29">
-        <f t="shared" si="2"/>
-        <v>8.99</v>
+        <f t="shared" si="1"/>
+        <v>5.99</v>
       </c>
       <c r="I29">
+        <f>ROUNDDOWN(D29*F29/$C$38, 0)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="5"/>
+      <c r="B30" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30">
+        <v>2</v>
+      </c>
+      <c r="D30">
+        <v>30</v>
+      </c>
+      <c r="E30">
+        <f>C30*$C$38</f>
+        <v>14</v>
+      </c>
+      <c r="F30">
         <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="G30">
+        <v>8.5399999999999991</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="1"/>
+        <v>8.5399999999999991</v>
+      </c>
+      <c r="I30">
+        <f>ROUNDDOWN(D30*F30/$C$38, 0)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="5"/>
+      <c r="B31" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31">
         <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B30" t="s">
-        <v>33</v>
-      </c>
-      <c r="C30">
-        <v>4</v>
-      </c>
-      <c r="D30">
-        <v>50</v>
-      </c>
-      <c r="E30">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="F30">
-        <f>ROUNDUP(E30/D30,0)</f>
-        <v>1</v>
-      </c>
-      <c r="G30">
-        <v>6.19</v>
-      </c>
-      <c r="H30">
-        <f t="shared" si="2"/>
-        <v>6.19</v>
-      </c>
-      <c r="I30">
-        <f t="shared" si="3"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B31" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31">
-        <v>6</v>
       </c>
       <c r="D31">
         <v>20</v>
       </c>
       <c r="E31">
-        <f t="shared" si="0"/>
-        <v>42</v>
+        <f>C31*$C$38</f>
+        <v>14</v>
       </c>
       <c r="F31">
-        <f t="shared" si="4"/>
-        <v>3</v>
+        <f t="shared" si="2"/>
+        <v>1</v>
       </c>
       <c r="G31">
-        <v>6.99</v>
+        <v>8.99</v>
       </c>
       <c r="H31">
-        <f t="shared" si="2"/>
-        <v>20.97</v>
+        <f t="shared" si="1"/>
+        <v>8.99</v>
       </c>
       <c r="I31">
-        <f t="shared" si="3"/>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="4"/>
+        <f>ROUNDDOWN(D31*F31/$C$38, 0)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>75</v>
+      </c>
       <c r="B32" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D32">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E32">
-        <f t="shared" si="0"/>
-        <v>7</v>
+        <f>C32*$C$38</f>
+        <v>28</v>
       </c>
       <c r="F32">
         <f>ROUNDUP(E32/D32,0)</f>
         <v>1</v>
       </c>
       <c r="G32">
+        <v>6.19</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="1"/>
+        <v>6.19</v>
+      </c>
+      <c r="I32">
+        <f>ROUNDDOWN(D32*F32/$C$38, 0)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33">
+        <v>6</v>
+      </c>
+      <c r="D33">
+        <v>20</v>
+      </c>
+      <c r="E33">
+        <f>C33*$C$38</f>
+        <v>42</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="G33">
+        <v>6.99</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="1"/>
+        <v>20.97</v>
+      </c>
+      <c r="I33">
+        <f>ROUNDDOWN(D33*F33/$C$38, 0)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="5"/>
+      <c r="B34" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>10</v>
+      </c>
+      <c r="E34">
+        <f>C34*$C$38</f>
+        <v>7</v>
+      </c>
+      <c r="F34">
+        <f>ROUNDUP(E34/D34,0)</f>
+        <v>1</v>
+      </c>
+      <c r="G34">
         <v>9.69</v>
       </c>
-      <c r="H32">
+      <c r="H34">
+        <f t="shared" si="1"/>
+        <v>9.69</v>
+      </c>
+      <c r="I34">
+        <f>ROUNDDOWN(D34*F34/$C$38, 0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="5"/>
+      <c r="B35" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35">
+        <v>20</v>
+      </c>
+      <c r="E35">
+        <f>C35*$C$38</f>
+        <v>7</v>
+      </c>
+      <c r="F35">
         <f t="shared" si="2"/>
-        <v>9.69</v>
-      </c>
-      <c r="I32">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="4"/>
-      <c r="B33" t="s">
-        <v>40</v>
-      </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-      <c r="D33">
-        <v>19</v>
-      </c>
-      <c r="E33">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="F33">
-        <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="G33">
-        <v>15.79</v>
-      </c>
-      <c r="H33">
-        <f t="shared" si="2"/>
-        <v>15.79</v>
-      </c>
-      <c r="I33">
-        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="G35">
+        <v>26</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="I35">
+        <f>ROUNDDOWN(D35*F35/$C$38, 0)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-      <c r="B34" t="s">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="5"/>
+      <c r="B36" t="s">
         <v>61</v>
       </c>
-      <c r="F34">
-        <v>1</v>
-      </c>
-      <c r="G34">
+      <c r="F36">
+        <v>1</v>
+      </c>
+      <c r="G36">
         <v>11.59</v>
       </c>
-      <c r="H34">
-        <f t="shared" si="2"/>
+      <c r="H36">
+        <f t="shared" si="1"/>
         <v>11.59</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
-        <v>45</v>
-      </c>
-      <c r="C36">
-        <f>SUM(C37:C39)</f>
-        <v>7</v>
-      </c>
-      <c r="G36" t="s">
-        <v>64</v>
-      </c>
-      <c r="H36">
-        <f>SUM(H2:H35)</f>
-        <v>310.94000000000005</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
-        <v>1</v>
-      </c>
-      <c r="C37">
-        <v>1</v>
-      </c>
-      <c r="G37" t="s">
-        <v>63</v>
-      </c>
-      <c r="H37">
-        <v>11.96</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="C38">
-        <v>3</v>
+        <f>SUM(C39:C41)</f>
+        <v>7</v>
       </c>
       <c r="G38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H38">
-        <f>H36+H37</f>
-        <v>322.90000000000003</v>
+        <f>SUM(H2:H37)</f>
+        <v>342.5200000000001</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="G39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H39">
+        <v>11.96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>0</v>
+      </c>
+      <c r="C40">
+        <v>3</v>
+      </c>
+      <c r="G40" t="s">
+        <v>65</v>
+      </c>
+      <c r="H40">
+        <f>H38+H39</f>
+        <v>354.48000000000008</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
         <v>69</v>
       </c>
-      <c r="C39">
+      <c r="C41">
         <v>3</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G41" t="s">
         <v>60</v>
       </c>
-      <c r="H39">
-        <f>H38/C36</f>
-        <v>46.128571428571433</v>
+      <c r="H41">
+        <f>H40/C38</f>
+        <v>50.640000000000008</v>
       </c>
     </row>
   </sheetData>
@@ -2025,8 +2110,8 @@
     <mergeCell ref="A2:A11"/>
     <mergeCell ref="A12:A18"/>
     <mergeCell ref="A19:A26"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="A33:A36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2034,14 +2119,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{844A380A-6B65-4EF5-8C07-FFBB17288005}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="44.42578125" customWidth="1"/>
     <col min="3" max="3" width="9.28515625" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" customWidth="1"/>
     <col min="5" max="5" width="34.5703125" customWidth="1"/>
-    <col min="6" max="6" width="79.5703125" customWidth="1"/>
+    <col min="6" max="6" width="93.85546875" customWidth="1"/>
     <col min="7" max="7" width="33.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2069,7 +2154,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>107</v>
       </c>
       <c r="B2" t="s">
@@ -2092,7 +2177,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
+      <c r="A3" s="4"/>
       <c r="B3" t="s">
         <v>81</v>
       </c>
@@ -2113,7 +2198,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
+      <c r="A4" s="4"/>
       <c r="B4" t="s">
         <v>19</v>
       </c>
@@ -2131,7 +2216,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
+      <c r="A5" s="4"/>
       <c r="B5" t="s">
         <v>122</v>
       </c>
@@ -2149,7 +2234,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
+      <c r="A6" s="4"/>
       <c r="B6" t="s">
         <v>136</v>
       </c>
@@ -2168,7 +2253,7 @@
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
@@ -2185,7 +2270,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
+      <c r="A8" s="6"/>
       <c r="B8" t="s">
         <v>9</v>
       </c>
@@ -2197,7 +2282,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B9" t="s">
@@ -2214,7 +2299,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="5"/>
+      <c r="A10" s="6"/>
       <c r="B10" t="s">
         <v>15</v>
       </c>
@@ -2226,7 +2311,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>76</v>
       </c>
       <c r="B11" t="s">
@@ -2240,7 +2325,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="5"/>
+      <c r="A12" s="6"/>
       <c r="B12" t="s">
         <v>67</v>
       </c>
@@ -2252,7 +2337,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
+      <c r="A13" s="6"/>
       <c r="B13" t="s">
         <v>31</v>
       </c>
@@ -2267,7 +2352,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="5"/>
+      <c r="A14" s="6"/>
       <c r="B14" t="s">
         <v>22</v>
       </c>
@@ -2282,14 +2367,14 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="5"/>
+      <c r="A15" s="6"/>
       <c r="B15" t="s">
         <v>143</v>
       </c>
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="5"/>
+      <c r="A16" s="6"/>
       <c r="B16" t="s">
         <v>144</v>
       </c>
@@ -2299,7 +2384,7 @@
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>119</v>
       </c>
       <c r="B17" t="s">
@@ -2319,7 +2404,7 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="5"/>
+      <c r="A18" s="6"/>
       <c r="B18" t="s">
         <v>24</v>
       </c>
@@ -2337,7 +2422,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="5"/>
+      <c r="A19" s="6"/>
       <c r="B19" t="s">
         <v>34</v>
       </c>
@@ -2378,6 +2463,23 @@
       </c>
       <c r="F23" t="s">
         <v>153</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>157</v>
+      </c>
+      <c r="B24" t="s">
+        <v>158</v>
+      </c>
+      <c r="C24">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <v>6</v>
+      </c>
+      <c r="F24" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>